<commit_message>
large park layout/scale fixes, park labels, July date, currentPct blank fix
</commit_message>
<xml_diff>
--- a/largepark_work/KPI PARKS GR.xlsx
+++ b/largepark_work/KPI PARKS GR.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\BPLA Dropbox\03 Planning\1232-T2-TM2_1-GIS-Remote-Sensing\06_GIS-Data\35_Projects Review\large_park\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saeed\Downloads\Aa_Canopy\largepark_work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3216E5E5-A054-46F6-AD4E-33E057144734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D042038-5C76-4A8B-BC08-57B0EEB6A2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{77722B99-B285-4C19-91B2-6CA9254EDB85}"/>
   </bookViews>
@@ -388,21 +388,21 @@
   <dxfs count="3">
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -838,7 +838,7 @@
         <v>4844</v>
       </c>
       <c r="F3" s="17">
-        <v>48305</v>
+        <v>69065</v>
       </c>
       <c r="G3" s="17">
         <v>12667</v>
@@ -862,15 +862,15 @@
       </c>
       <c r="M3" s="8">
         <f>100/B3*F3</f>
-        <v>41.027187253161657</v>
+        <v>58.659407672903626</v>
       </c>
       <c r="N3" s="8">
         <f>100/B3*(F3+J3)</f>
-        <v>46.708397387441714</v>
-      </c>
-      <c r="O3" s="9" t="e">
+        <v>64.340617807183691</v>
+      </c>
+      <c r="O3" s="9">
         <f t="shared" ref="O3:O6" si="0">IF(M3&gt;K3,0,(W3/V3))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -881,7 +881,7 @@
         <v>147378</v>
       </c>
       <c r="C4" s="17">
-        <v>27471</v>
+        <v>74470</v>
       </c>
       <c r="D4" s="17">
         <v>3228</v>
@@ -890,7 +890,7 @@
         <v>10112</v>
       </c>
       <c r="F4" s="17">
-        <v>72988</v>
+        <v>105987</v>
       </c>
       <c r="G4" s="17">
         <v>1482</v>
@@ -914,15 +914,15 @@
       </c>
       <c r="M4" s="10">
         <f t="shared" ref="M4:M7" si="3">100/B4*F4</f>
-        <v>49.524352345668966</v>
+        <v>71.915075520091193</v>
       </c>
       <c r="N4" s="10">
         <f>100/B4*(F4+J4)</f>
-        <v>49.641737572772058</v>
-      </c>
-      <c r="O4" s="11" t="e">
+        <v>72.032460747194293</v>
+      </c>
+      <c r="O4" s="11">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -942,7 +942,7 @@
         <v>7332</v>
       </c>
       <c r="F5" s="17">
-        <v>49255</v>
+        <v>53681</v>
       </c>
       <c r="G5" s="17">
         <v>5334</v>
@@ -966,11 +966,11 @@
       </c>
       <c r="M5" s="10">
         <f t="shared" si="3"/>
-        <v>38.103010799269732</v>
+        <v>41.526905343936626</v>
       </c>
       <c r="N5" s="10">
         <f t="shared" ref="N5:N7" si="4">100/B5*(F5+J5)</f>
-        <v>40.127487081102828</v>
+        <v>43.551381625769721</v>
       </c>
       <c r="O5" s="11" t="e">
         <f t="shared" si="0"/>
@@ -994,7 +994,7 @@
         <v>2519</v>
       </c>
       <c r="F6" s="17">
-        <v>18523</v>
+        <v>31909</v>
       </c>
       <c r="G6" s="17">
         <v>2876</v>
@@ -1018,15 +1018,15 @@
       </c>
       <c r="M6" s="10">
         <f t="shared" si="3"/>
-        <v>34.45306251511262</v>
+        <v>59.351226680058772</v>
       </c>
       <c r="N6" s="10">
         <f t="shared" si="4"/>
-        <v>36.846902144597586</v>
-      </c>
-      <c r="O6" s="11" t="e">
+        <v>61.745066309543738</v>
+      </c>
+      <c r="O6" s="11">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1086,7 +1086,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="L3:L7">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -1107,12 +1107,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L3:N7">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
       <formula>$K$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M3:M6">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Update Bader KPI data after current canopy replacement
</commit_message>
<xml_diff>
--- a/largepark_work/KPI PARKS GR.xlsx
+++ b/largepark_work/KPI PARKS GR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saeed\Downloads\Aa_Canopy\largepark_work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D042038-5C76-4A8B-BC08-57B0EEB6A2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1834706D-E71F-49A2-ADFC-732A3FF4BD31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{77722B99-B285-4C19-91B2-6CA9254EDB85}"/>
   </bookViews>
@@ -388,21 +388,21 @@
   <dxfs count="3">
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1034,47 +1034,47 @@
         <v>20</v>
       </c>
       <c r="B7" s="23">
-        <v>172756</v>
+        <v>172745</v>
       </c>
       <c r="C7" s="20">
-        <v>9058</v>
+        <v>12866</v>
       </c>
       <c r="D7" s="20">
-        <v>1386</v>
+        <v>1377</v>
       </c>
       <c r="E7" s="20">
-        <v>4349</v>
+        <v>1345</v>
       </c>
       <c r="F7" s="20">
-        <v>8338</v>
+        <v>76114</v>
       </c>
       <c r="G7" s="20">
-        <v>9058</v>
+        <v>6479</v>
       </c>
       <c r="H7" s="18">
-        <v>31</v>
+        <v>293</v>
       </c>
       <c r="I7" s="18">
-        <f t="shared" si="1"/>
-        <v>1417</v>
+        <f>H7+D7</f>
+        <v>1670</v>
       </c>
       <c r="J7" s="18">
-        <v>1497</v>
+        <v>7748</v>
       </c>
       <c r="K7" s="14">
         <v>50</v>
       </c>
       <c r="L7" s="10">
         <f t="shared" si="2"/>
-        <v>2.5174234179999537</v>
+        <v>0.77860430113751489</v>
       </c>
       <c r="M7" s="10">
         <f t="shared" si="3"/>
-        <v>4.8264604413160752</v>
+        <v>44.061477900952269</v>
       </c>
       <c r="N7" s="10">
         <f t="shared" si="4"/>
-        <v>5.6930005325430084</v>
+        <v>48.546701785869345</v>
       </c>
       <c r="O7" s="11" t="e">
         <f>IF(M7&gt;K7,0,(W7/V7))</f>
@@ -1086,7 +1086,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="L3:L7">
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
     <cfRule type="colorScale" priority="4">
@@ -1107,12 +1107,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L3:N7">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
       <formula>$K$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M3:M6">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>$K$3</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>